<commit_message>
actualizacion tablas validacion stage1
</commit_message>
<xml_diff>
--- a/tfm_key_experiments_comparison.xlsx
+++ b/tfm_key_experiments_comparison.xlsx
@@ -9,18 +9,20 @@
   <sheets>
     <sheet name="Lectura_rapida" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Stage1_TEST_interno" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stage1_externo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Stage2_VALIDATION" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Stage2_TEST_final" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Definiciones" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Stage1_VALIDATION" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stage1_externo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Stage2_VALIDATION" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Stage2_TEST_final" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Definiciones" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lectura_rapida'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage1_TEST_interno'!$A$1:$AA$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage1_externo'!$A$1:$U$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stage2_VALIDATION'!$A$1:$X$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Stage2_TEST_final'!$A$1:$W$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Definiciones'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage1_TEST_interno'!$A$1:$AO$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage1_VALIDATION'!$A$1:$Z$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stage1_externo'!$A$1:$U$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Stage2_VALIDATION'!$A$1:$X$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Stage2_TEST_final'!$A$1:$W$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Definiciones'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,9 +182,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TFMTable2" displayName="TFMTable2" ref="A1:AA6" headerRowCount="1">
-  <autoFilter ref="A1:AA6"/>
-  <tableColumns count="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TFMTable2" displayName="TFMTable2" ref="A1:AO6" headerRowCount="1">
+  <autoFilter ref="A1:AO6"/>
+  <tableColumns count="41">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Experimento"/>
     <tableColumn id="3" name="Datos positivos"/>
@@ -191,32 +193,81 @@
     <tableColumn id="6" name="Grupo de comparabilidad"/>
     <tableColumn id="7" name="Configuración LR"/>
     <tableColumn id="8" name="Umbral"/>
-    <tableColumn id="9" name="N TEST"/>
-    <tableColumn id="10" name="No tos TEST"/>
-    <tableColumn id="11" name="Tos TEST"/>
-    <tableColumn id="12" name="Accuracy TEST"/>
-    <tableColumn id="13" name="Balanced accuracy TEST"/>
-    <tableColumn id="14" name="Sensibilidad / recall tos TEST"/>
-    <tableColumn id="15" name="Especificidad / recall no tos TEST"/>
-    <tableColumn id="16" name="Precisión tos TEST"/>
-    <tableColumn id="17" name="F1 tos TEST"/>
-    <tableColumn id="18" name="Macro-F1 TEST"/>
-    <tableColumn id="19" name="ROC-AUC TEST"/>
-    <tableColumn id="20" name="Recall toses CoughVID TEST"/>
-    <tableColumn id="21" name="Recall toses FSD50K TEST"/>
-    <tableColumn id="22" name="FP TEST"/>
-    <tableColumn id="23" name="FN TEST"/>
-    <tableColumn id="24" name="Macro-F1 OOF"/>
-    <tableColumn id="25" name="Macro-F1 VALIDATION"/>
-    <tableColumn id="26" name="Modelo KB"/>
-    <tableColumn id="27" name="Fuente"/>
+    <tableColumn id="9" name="N VALIDATION"/>
+    <tableColumn id="10" name="No tos VALIDATION"/>
+    <tableColumn id="11" name="Tos VALIDATION"/>
+    <tableColumn id="12" name="Accuracy VALIDATION"/>
+    <tableColumn id="13" name="Balanced accuracy VALIDATION"/>
+    <tableColumn id="14" name="Sensibilidad / recall tos VALIDATION"/>
+    <tableColumn id="15" name="Especificidad / recall no tos VALIDATION"/>
+    <tableColumn id="16" name="Precision tos VALIDATION"/>
+    <tableColumn id="17" name="F1 tos VALIDATION"/>
+    <tableColumn id="18" name="Macro-F1 VALIDATION"/>
+    <tableColumn id="19" name="ROC-AUC VALIDATION"/>
+    <tableColumn id="20" name="TN VALIDATION"/>
+    <tableColumn id="21" name="FP VALIDATION"/>
+    <tableColumn id="22" name="FN VALIDATION"/>
+    <tableColumn id="23" name="TP VALIDATION"/>
+    <tableColumn id="24" name="N TEST"/>
+    <tableColumn id="25" name="No tos TEST"/>
+    <tableColumn id="26" name="Tos TEST"/>
+    <tableColumn id="27" name="Accuracy TEST"/>
+    <tableColumn id="28" name="Balanced accuracy TEST"/>
+    <tableColumn id="29" name="Sensibilidad / recall tos TEST"/>
+    <tableColumn id="30" name="Especificidad / recall no tos TEST"/>
+    <tableColumn id="31" name="Precisión tos TEST"/>
+    <tableColumn id="32" name="F1 tos TEST"/>
+    <tableColumn id="33" name="Macro-F1 TEST"/>
+    <tableColumn id="34" name="ROC-AUC TEST"/>
+    <tableColumn id="35" name="Recall toses CoughVID TEST"/>
+    <tableColumn id="36" name="Recall toses FSD50K TEST"/>
+    <tableColumn id="37" name="FP TEST"/>
+    <tableColumn id="38" name="FN TEST"/>
+    <tableColumn id="39" name="Macro-F1 OOF"/>
+    <tableColumn id="40" name="Modelo KB"/>
+    <tableColumn id="41" name="Fuente"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TFMTable3" displayName="TFMTable3" ref="A1:U4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TFMTable3" displayName="TFMTable3" ref="A1:Z6" headerRowCount="1">
+  <autoFilter ref="A1:Z6"/>
+  <tableColumns count="26">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Experimento"/>
+    <tableColumn id="3" name="Datos positivos"/>
+    <tableColumn id="4" name="Augmentation en TRAIN"/>
+    <tableColumn id="5" name="Protocolo"/>
+    <tableColumn id="6" name="Grupo de comparabilidad"/>
+    <tableColumn id="7" name="Configuración LR"/>
+    <tableColumn id="8" name="Umbral"/>
+    <tableColumn id="9" name="N VALIDATION"/>
+    <tableColumn id="10" name="No tos VALIDATION"/>
+    <tableColumn id="11" name="Tos VALIDATION"/>
+    <tableColumn id="12" name="Accuracy VALIDATION"/>
+    <tableColumn id="13" name="Balanced accuracy VALIDATION"/>
+    <tableColumn id="14" name="Sensibilidad / recall tos VALIDATION"/>
+    <tableColumn id="15" name="Especificidad / recall no tos VALIDATION"/>
+    <tableColumn id="16" name="Precision tos VALIDATION"/>
+    <tableColumn id="17" name="F1 tos VALIDATION"/>
+    <tableColumn id="18" name="Macro-F1 VALIDATION"/>
+    <tableColumn id="19" name="ROC-AUC VALIDATION"/>
+    <tableColumn id="20" name="TN VALIDATION"/>
+    <tableColumn id="21" name="FP VALIDATION"/>
+    <tableColumn id="22" name="FN VALIDATION"/>
+    <tableColumn id="23" name="TP VALIDATION"/>
+    <tableColumn id="24" name="Macro-F1 OOF"/>
+    <tableColumn id="25" name="Modelo KB"/>
+    <tableColumn id="26" name="Fuente"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TFMTable4" displayName="TFMTable4" ref="A1:U4" headerRowCount="1">
   <autoFilter ref="A1:U4"/>
   <tableColumns count="21">
     <tableColumn id="1" name="ID"/>
@@ -245,8 +296,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TFMTable4" displayName="TFMTable4" ref="A1:X12" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TFMTable5" displayName="TFMTable5" ref="A1:X12" headerRowCount="1">
   <autoFilter ref="A1:X12"/>
   <tableColumns count="24">
     <tableColumn id="1" name="ID"/>
@@ -278,9 +329,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TFMTable5" displayName="TFMTable5" ref="A1:W2" headerRowCount="1">
-  <autoFilter ref="A1:W2"/>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TFMTable6" displayName="TFMTable6" ref="A1:W5" headerRowCount="1">
+  <autoFilter ref="A1:W5"/>
   <tableColumns count="23">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Experimento"/>
@@ -310,8 +361,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TFMTable6" displayName="TFMTable6" ref="A1:B10" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TFMTable7" displayName="TFMTable7" ref="A1:B10" headerRowCount="1">
   <autoFilter ref="A1:B10"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Concepto"/>
@@ -697,7 +748,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>El WST+LR congelado obtiene macro-F1 0.5942, sensibilidad wet 0.4750, especificidad dry 0.7425 y ROC-AUC 0.6999.</t>
+          <t>Con los cuatro modelos congelados sobre el mismo TEST, la late fusion obtiene el mayor macro-F1 (0.6751), balanced accuracy (0.6729) y ROC-AUC (0.7220). Log-Mel alcanza el mayor recall wet (0.5500). WST-LR mejora modestamente al baseline MFCC-LR.</t>
         </is>
       </c>
     </row>
@@ -716,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AO6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -727,25 +778,39 @@
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="26" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="21" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="38" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="32" customWidth="1" min="29" max="29"/>
+    <col width="36" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="28" customWidth="1" min="35" max="35"/>
+    <col width="26" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="37" max="37"/>
+    <col width="11" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="14" customWidth="1" min="40" max="40"/>
+    <col width="38" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -791,95 +856,165 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>N VALIDATION</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>No tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy VALIDATION</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Balanced accuracy VALIDATION</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Sensibilidad / recall tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Especificidad / recall no tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Precision tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>F1 tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1 VALIDATION</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>ROC-AUC VALIDATION</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>TN VALIDATION</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>FP VALIDATION</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>FN VALIDATION</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>TP VALIDATION</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
           <t>N TEST</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>No tos TEST</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>Tos TEST</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Accuracy TEST</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>Balanced accuracy TEST</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>Sensibilidad / recall tos TEST</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>Especificidad / recall no tos TEST</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>Precisión tos TEST</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>F1 tos TEST</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>Macro-F1 TEST</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>ROC-AUC TEST</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>Recall toses CoughVID TEST</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>Recall toses FSD50K TEST</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>FP TEST</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>FN TEST</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>Macro-F1 OOF</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>Macro-F1 VALIDATION</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>Modelo KB</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -925,58 +1060,100 @@
         <v>0.5</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1642</v>
+        <v>1640</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>1219</v>
+        <v>1217</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>423</v>
       </c>
       <c r="L2" s="4" t="n">
+        <v>0.9810975609756096</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0.9772383355575368</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0.9692671394799054</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0.9852095316351684</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0.9579439252336448</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0.963572267920094</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>0.9754049071177252</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.9956292942184304</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>1199</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>410</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>1642</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>1219</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>423</v>
+      </c>
+      <c r="AA2" s="4" t="n">
         <v>0.9811205846528624</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="AB2" s="4" t="n">
         <v>0.9749348863638568</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="AC2" s="4" t="n">
         <v>0.9621749408983452</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="AD2" s="4" t="n">
         <v>0.9876948318293683</v>
       </c>
-      <c r="P2" s="4" t="n">
+      <c r="AE2" s="4" t="n">
         <v>0.9644549763033176</v>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="AF2" s="4" t="n">
         <v>0.9633136094674556</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="AG2" s="4" t="n">
         <v>0.9753017411830922</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="AH2" s="4" t="n">
         <v>0.9984000372354972</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="AI2" s="4" t="n">
         <v>0.9621749408983452</v>
       </c>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="3" t="n">
+      <c r="AJ2" s="4" t="inlineStr"/>
+      <c r="AK2" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="AL2" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="AM2" s="4" t="n">
         <v>0.9743136202185564</v>
       </c>
-      <c r="Y2" s="4" t="n">
-        <v>0.9754049071177252</v>
-      </c>
-      <c r="Z2" s="3" t="n">
+      <c r="AN2" s="3" t="n">
         <v>4.9970703125</v>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>results_stage1_cough_no_cough\mfcc117_lr_random\full\metrics_summary.csv</t>
         </is>
@@ -1022,60 +1199,102 @@
         <v>0.5</v>
       </c>
       <c r="I3" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.9713282621416032</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.9599781937188204</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0.9352051835853132</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.9847512038523274</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>0.9579646017699116</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.946448087431694</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0.963435789620761</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.9932553068306702</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>1227</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>433</v>
+      </c>
+      <c r="X3" s="3" t="n">
         <v>1689</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="Y3" s="3" t="n">
         <v>1261</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="Z3" s="3" t="n">
         <v>428</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="AA3" s="4" t="n">
         <v>0.9692125518058022</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="AB3" s="4" t="n">
         <v>0.9608603170603364</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="AC3" s="4" t="n">
         <v>0.9439252336448598</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="AD3" s="4" t="n">
         <v>0.9777954004758128</v>
       </c>
-      <c r="P3" s="4" t="n">
+      <c r="AE3" s="4" t="n">
         <v>0.9351851851851852</v>
       </c>
-      <c r="Q3" s="4" t="n">
+      <c r="AF3" s="4" t="n">
         <v>0.9395348837209302</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="AG3" s="4" t="n">
         <v>0.9594417865784952</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="AH3" s="4" t="n">
         <v>0.9935020418448496</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="AI3" s="4" t="n">
         <v>0.977667493796526</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="AJ3" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="V3" s="3" t="n">
+      <c r="AK3" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="W3" s="3" t="n">
+      <c r="AL3" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="X3" s="4" t="n">
+      <c r="AM3" s="4" t="n">
         <v>0.9544231772476612</v>
       </c>
-      <c r="Y3" s="4" t="n">
-        <v>0.963435789620761</v>
-      </c>
-      <c r="Z3" s="3" t="n">
+      <c r="AN3" s="3" t="n">
         <v>4.9970703125</v>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AO3" s="3" t="inlineStr">
         <is>
           <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_random\full\metrics_summary.csv</t>
         </is>
@@ -1121,60 +1340,102 @@
         <v>0.5</v>
       </c>
       <c r="I4" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0.9379754242246928</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0.9493203304570306</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0.9740820734341252</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.9245585874799358</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0.8275229357798165</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0.8948412698412699</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0.9254289336758216</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.9900120991925784</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>1152</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>451</v>
+      </c>
+      <c r="X4" s="3" t="n">
         <v>1689</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="Y4" s="3" t="n">
         <v>1261</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="Z4" s="3" t="n">
         <v>428</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="AA4" s="4" t="n">
         <v>0.9396092362344582</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="AB4" s="4" t="n">
         <v>0.9533821992633054</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="AC4" s="4" t="n">
         <v>0.9813084112149532</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="AD4" s="4" t="n">
         <v>0.9254559873116576</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="AE4" s="4" t="n">
         <v>0.8171206225680934</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="AF4" s="4" t="n">
         <v>0.89171974522293</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="AG4" s="4" t="n">
         <v>0.924923912020332</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="AH4" s="4" t="n">
         <v>0.9917307136451564</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="AI4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="AJ4" s="4" t="n">
         <v>0.68</v>
       </c>
-      <c r="V4" s="3" t="n">
+      <c r="AK4" s="3" t="n">
         <v>94</v>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="AL4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="X4" s="4" t="n">
+      <c r="AM4" s="4" t="n">
         <v>0.9221817270697834</v>
       </c>
-      <c r="Y4" s="4" t="n">
-        <v>0.9254289336758216</v>
-      </c>
-      <c r="Z4" s="3" t="n">
+      <c r="AN4" s="3" t="n">
         <v>4.9970703125</v>
       </c>
-      <c r="AA4" s="3" t="inlineStr">
+      <c r="AO4" s="3" t="inlineStr">
         <is>
           <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_audio_aug_random\full\metrics_summary.csv</t>
         </is>
@@ -1220,60 +1481,102 @@
         <v>0.5</v>
       </c>
       <c r="I5" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.946167349327092</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.9515451604963095</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0.9632829373650108</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0.9398073836276084</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>0.8560460652591171</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.9065040650406504</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0.9343531007208182</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.9884971000072804</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>1171</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>446</v>
+      </c>
+      <c r="X5" s="3" t="n">
         <v>1689</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="Y5" s="3" t="n">
         <v>1261</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="Z5" s="3" t="n">
         <v>428</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="AA5" s="4" t="n">
         <v>0.9561870929544108</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="AB5" s="4" t="n">
         <v>0.9613976446522934</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="AC5" s="4" t="n">
         <v>0.97196261682243</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="AD5" s="4" t="n">
         <v>0.950832672482157</v>
       </c>
-      <c r="P5" s="4" t="n">
+      <c r="AE5" s="4" t="n">
         <v>0.8702928870292888</v>
       </c>
-      <c r="Q5" s="4" t="n">
+      <c r="AF5" s="4" t="n">
         <v>0.9183222958057397</v>
       </c>
-      <c r="R5" s="4" t="n">
+      <c r="AG5" s="4" t="n">
         <v>0.9441935103624168</v>
       </c>
-      <c r="S5" s="4" t="n">
+      <c r="AH5" s="4" t="n">
         <v>0.9899297397852173</v>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="AI5" s="4" t="n">
         <v>0.9975186104218362</v>
       </c>
-      <c r="U5" s="4" t="n">
+      <c r="AJ5" s="4" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="V5" s="3" t="n">
+      <c r="AK5" s="3" t="n">
         <v>62</v>
       </c>
-      <c r="W5" s="3" t="n">
+      <c r="AL5" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="X5" s="4" t="n">
+      <c r="AM5" s="4" t="n">
         <v>0.9290377500221316</v>
       </c>
-      <c r="Y5" s="4" t="n">
-        <v>0.9343531007208182</v>
-      </c>
-      <c r="Z5" s="3" t="n">
+      <c r="AN5" s="3" t="n">
         <v>4.9970703125</v>
       </c>
-      <c r="AA5" s="3" t="inlineStr">
+      <c r="AO5" s="3" t="inlineStr">
         <is>
           <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_noise_aug_random\full\metrics_summary.csv</t>
         </is>
@@ -1319,65 +1622,107 @@
         <v>0.5</v>
       </c>
       <c r="I6" s="3" t="n">
+        <v>1705</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1212</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>493</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0.960117302052786</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0.9538974688543904</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0.9391480730223124</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0.9686468646864688</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0.9241516966067864</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0.93158953722334</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0.9517219209295508</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.9865208630396508</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>1174</v>
+      </c>
+      <c r="U6" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="X6" s="3" t="n">
         <v>1486</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="Y6" s="3" t="n">
         <v>1216</v>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="Z6" s="3" t="n">
         <v>270</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="AA6" s="4" t="n">
         <v>0.9582772543741588</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="AB6" s="4" t="n">
         <v>0.9500152290448344</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="AC6" s="4" t="n">
         <v>0.937037037037037</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="AD6" s="4" t="n">
         <v>0.9629934210526316</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="AE6" s="4" t="n">
         <v>0.8489932885906041</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="AF6" s="4" t="n">
         <v>0.8908450704225352</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="AG6" s="4" t="n">
         <v>0.932527360502449</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="AH6" s="4" t="n">
         <v>0.9911245126705652</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="AI6" s="4" t="n">
         <v>0.937037037037037</v>
       </c>
-      <c r="U6" s="4" t="inlineStr"/>
-      <c r="V6" s="3" t="n">
+      <c r="AJ6" s="4" t="inlineStr"/>
+      <c r="AK6" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="W6" s="3" t="n">
+      <c r="AL6" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="X6" s="4" t="n">
+      <c r="AM6" s="4" t="n">
         <v>0.9561967063357104</v>
       </c>
-      <c r="Y6" s="4" t="n">
-        <v>0.9517219209295508</v>
-      </c>
-      <c r="Z6" s="3" t="n">
+      <c r="AN6" s="3" t="n">
         <v>4.9970703125</v>
       </c>
-      <c r="AA6" s="3" t="inlineStr">
+      <c r="AO6" s="3" t="inlineStr">
         <is>
           <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_audio_quality_poor\full\metrics_summary.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA6"/>
+  <autoFilter ref="A1:AO6"/>
   <conditionalFormatting sqref="H2:H6">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -1438,7 +1783,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P6">
+  <conditionalFormatting sqref="Q2:Q6">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -1450,7 +1795,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q6">
+  <conditionalFormatting sqref="R2:R6">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -1462,7 +1807,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R6">
+  <conditionalFormatting sqref="S2:S6">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -1474,7 +1819,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S6">
+  <conditionalFormatting sqref="AA2:AA6">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -1486,7 +1831,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T6">
+  <conditionalFormatting sqref="AB2:AB6">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -1498,7 +1843,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U6">
+  <conditionalFormatting sqref="AC2:AC6">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1510,7 +1855,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X6">
+  <conditionalFormatting sqref="AD2:AD6">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -1522,8 +1867,80 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y2:Y6">
+  <conditionalFormatting sqref="AE2:AE6">
     <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF2:AF6">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG2:AG6">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AH2:AH6">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI2:AI6">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ2:AJ6">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM2:AM6">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1542,6 +1959,772 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="38" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Experimento</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Datos positivos</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Augmentation en TRAIN</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Grupo de comparabilidad</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Configuración LR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Umbral</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>N VALIDATION</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>No tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy VALIDATION</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Balanced accuracy VALIDATION</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Sensibilidad / recall tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Especificidad / recall no tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Precision tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>F1 tos VALIDATION</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1 VALIDATION</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>ROC-AUC VALIDATION</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>TN VALIDATION</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>FP VALIDATION</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>FN VALIDATION</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>TP VALIDATION</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1 OOF</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>Modelo KB</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>S1-LR-01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + LR; CoughVID como clase positiva</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>CoughVID</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Split aleatorio agrupado</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>A: referencia anterior; distinto conjunto positivo</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>lr__C0p3__l1__weight_none</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>1640</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>1217</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>423</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0.9810975609756096</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0.9772383355575368</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0.9692671394799054</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0.9852095316351684</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0.9579439252336448</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0.963572267920094</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>0.9754049071177252</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.9956292942184304</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>1199</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>410</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.9743136202185564</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>4.9970703125</v>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>results_stage1_cough_no_cough\mfcc117_lr_random\full\metrics_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S1-LR-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + LR; CoughVID + FSD50K</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>CoughVID + toses FSD50K revisadas y segmentadas</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Split aleatorio agrupado</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>B: comparación principal; mismo TEST que S1-LR-03/04</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>lr__C0p3__l1__weight_none</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.9713282621416032</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.9599781937188204</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0.9352051835853132</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.9847512038523274</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>0.9579646017699116</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.946448087431694</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0.963435789620761</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.9932553068306702</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>1227</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>433</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.9544231772476612</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>4.9970703125</v>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_random\full\metrics_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>S1-LR-03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + LR; augmentation pitch + ruido</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>CoughVID + toses FSD50K revisadas y segmentadas</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2 variantes/tos TRAIN: pitch ±1.5 o ruido moderado/alto</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Split aleatorio agrupado; OOF/VAL/TEST solo originales</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>B: comparación principal; mismo TEST que S1-LR-02/04</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>lr__C0p3__l1__weight_none</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0.9379754242246928</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0.9493203304570306</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0.9740820734341252</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.9245585874799358</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0.8275229357798165</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0.8948412698412699</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0.9254289336758216</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.9900120991925784</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>1152</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>451</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0.9221817270697834</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>4.9970703125</v>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_audio_aug_random\full\metrics_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>S1-LR-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + LR; augmentation solo ruido</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CoughVID + toses FSD50K revisadas y segmentadas</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1 variante/tos TRAIN: mezcla a 10 o 20 dB SNR</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Split aleatorio agrupado; OOF/VAL/TEST solo originales</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>B: comparación principal; mismo TEST que S1-LR-02/03</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>lr__C0p3__l1__weight_none</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1246</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.946167349327092</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.9515451604963095</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0.9632829373650108</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0.9398073836276084</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>0.8560460652591171</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.9065040650406504</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0.9343531007208182</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.9884971000072804</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>1171</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>446</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0.9290377500221316</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>4.9970703125</v>
+      </c>
+      <c r="Z5" s="3" t="inlineStr">
+        <is>
+          <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_noise_aug_random\full\metrics_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>S1-LR-05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + LR; stress test de calidad poor</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>TRAIN/VAL: CoughVID + FSD50K; TEST: CoughVID poor</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Todas las toses CoughVID poor reservadas en TEST</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>C: análisis secundario de robustez; TEST diferente</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>lr__C0p3__l1__weight_none</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>1705</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1212</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>493</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0.960117302052786</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0.9538974688543904</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0.9391480730223124</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0.9686468646864688</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0.9241516966067864</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0.93158953722334</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0.9517219209295508</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.9865208630396508</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>1174</v>
+      </c>
+      <c r="U6" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>463</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0.9561967063357104</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>4.9970703125</v>
+      </c>
+      <c r="Z6" s="3" t="inlineStr">
+        <is>
+          <t>results_stage1_cough_no_cough\mfcc117_lr_fsd50k_cough_segments_audio_quality_poor\full\metrics_summary.csv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Z6"/>
+  <conditionalFormatting sqref="H2:H6">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L6">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M6">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N6">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2:O6">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q6">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R6">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S6">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X2:X6">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2028,7 +3211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3338,17 +4521,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -3368,7 +4551,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
     <col width="38" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
@@ -3492,26 +4675,26 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>WST recording + LR; búsqueda en dos fases</t>
+          <t>Late fusion WST-LR + Log-Mel CNN</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>TEST final tras congelar configuración y umbral mediante OOF; no usado para selección</t>
+          <t>Mismo TEST final; modelos, configuración, fusión y umbrales congelados mediante OOF antes de evaluarlo</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>logistic_regression__C0.001__pca128__no_whiten__gold1__wetcost1</t>
+          <t>late_fusion_wst_logmel_cnn__max_macro_f1__alpha0p35</t>
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.5451205759080889</v>
+        <v>0.5749472549246547</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>348</v>
@@ -3523,55 +4706,418 @@
         <v>80</v>
       </c>
       <c r="I2" s="4" t="n">
+        <v>0.7729885057471264</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.6728544776119403</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.4875</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0.8582089552238806</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0.5064935064935064</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0.4968152866242038</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0.6751237843139573</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0.7219682835820895</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0.4339878366714639</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>1089.7099609375</v>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>results_stage2_late_fusion_wst_logmel_cnn\full\stage2_test_model_comparison.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Log-Mel + tiny CNN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Mismo TEST final; modelos, configuración, fusión y umbrales congelados mediante OOF antes de evaluarlo</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>small__f16x32x64__dense32__drop0p3__l20p0005__lr0p0005</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.5510583445429802</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.7327586206896551</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.6686567164179105</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.7873134328358209</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.4356435643564356</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0.4861878453038674</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.6528026605160113</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0.7040111940298508</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.386390204604938</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>211</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>128.57421875</v>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>results_stage2_late_fusion_wst_logmel_cnn\full\stage2_test_model_comparison.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>WST recording + PCA128 + LR</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Mismo TEST final; modelos, configuración, fusión y umbrales congelados mediante OOF antes de evaluarlo</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>logistic_regression__C0.001__pca128__no_whiten__gold1__wetcost1</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.5451205759080889</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>0.6810344827586207</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>0.6087686567164179</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>0.475</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>0.7425373134328358</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>0.3551401869158878</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>0.4064171122994652</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>0.5941712280554301</v>
       </c>
-      <c r="P2" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>0.6998600746268657</v>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>0.4390574628533851</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="R4" s="3" t="n">
         <v>199</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="S4" s="3" t="n">
         <v>69</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="T4" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="U4" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V2" s="3" t="n">
+      <c r="V4" s="3" t="n">
         <v>961.146484375</v>
       </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>results_stage2_dry_wet_wst_recording_lr_two_phase_search\paper_q8_q1_t500_full\full\metrics_summary.csv</t>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>results_stage2_late_fusion_wst_logmel_cnn\full\stage2_test_model_comparison.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>MFCC117 + PCA128 + LR</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Mismo TEST final; modelos, configuración, fusión y umbrales congelados mediante OOF antes de evaluarlo</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>logistic_regression__C10__pca128</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.5829386662229422</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.6637931034482759</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.5975746268656716</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.7201492537313433</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.336283185840708</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0.3937823834196892</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0.580589004831117</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.6613339552238806</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.3718492859662215</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>179.291015625</v>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>results_stage2_late_fusion_wst_logmel_cnn\full\stage2_test_model_comparison.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W2"/>
+  <autoFilter ref="A1:W5"/>
+  <conditionalFormatting sqref="E2:E5">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I5">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J5">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K5">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L5">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M5">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N5">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2:O5">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:P5">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q5">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3579,7 +5125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>